<commit_message>
Cập nhật Thời khóa biểu giáo viên từ file 'TKB toàn trường CHECK - chuẩn.xlsx'
</commit_message>
<xml_diff>
--- a/Thời khóa biểu giáo viên/Thời khóa biểu - Cô Tân.xlsx
+++ b/Thời khóa biểu giáo viên/Thời khóa biểu - Cô Tân.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,22 +28,16 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="13"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Times New Roman"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
+      <i val="1"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -56,14 +50,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F497D"/>
-        <bgColor rgb="001F497D"/>
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,37 +71,46 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,309 +476,341 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUỔI</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>TIẾT</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>THỨ 2</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>THỨ 3</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>THỨ 4</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>THỨ 5</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>THỨ 6</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>THỨ 7</t>
+          <t>TRƯỜNG TIỂU HỌC VÀ THCS UNIGO</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SÁNG</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
+          <t>THỜI KHOÁ BIỂU CÁ NHÂN GIÁO VIÊN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Giáo viên: Cô Tân | Bộ môn: Toán | Tổng số: 24 tiết/tuần (Theo TKB toàn trường CHECK - chuẩn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Buổi / Tiết</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Thứ Hai</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Thứ Ba</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Thứ Tư</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Thứ Năm</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Thứ Sáu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>BUỔI SÁNG</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Tiết 1</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Tiết 2</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Tiết 3</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Tiết 4</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Tiết 5</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>CHIỀU</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>BUỔI CHIỀU</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Tiết 1</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Tiết 2</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 7A1</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(7A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Tiết 3</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Tiết 4</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 6A1</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Toán - 8A1</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(6A1)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Toán
+(8A1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Tiết 5</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="A2:A6"/>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cập nhật Thời khóa biểu toàn bộ giáo viên tại Hệ thống mẫu văn bản và Thời khóa biểu giáo viên từ TKB toàn trường CHECK - chuẩn.xlsx
</commit_message>
<xml_diff>
--- a/Thời khóa biểu giáo viên/Thời khóa biểu - Cô Tân.xlsx
+++ b/Thời khóa biểu giáo viên/Thời khóa biểu - Cô Tân.xlsx
@@ -560,20 +560,17 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
       <c r="E7" s="8" t="n"/>
@@ -588,21 +585,18 @@
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
     </row>
@@ -614,8 +608,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
       <c r="C9" s="8" t="n"/>
@@ -623,8 +616,7 @@
       <c r="E9" s="8" t="n"/>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
     </row>
@@ -648,21 +640,18 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
       <c r="D11" s="8" t="n"/>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
       <c r="F11" s="8" t="n"/>
@@ -687,32 +676,27 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
     </row>
@@ -725,21 +709,18 @@
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(7A1)</t>
+          <t>Toán (7A1)</t>
         </is>
       </c>
     </row>
@@ -755,8 +736,7 @@
       <c r="E15" s="8" t="n"/>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
     </row>
@@ -769,26 +749,22 @@
       <c r="B16" s="8" t="n"/>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(6A1)</t>
+          <t>Toán (6A1)</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Toán
-(8A1)</t>
+          <t>Toán (8A1)</t>
         </is>
       </c>
     </row>

</xml_diff>